<commit_message>
Panel de Director y regional carga de requisitos
</commit_message>
<xml_diff>
--- a/Archivos Excel/carga_requisitos_clase_Amigo.xlsx
+++ b/Archivos Excel/carga_requisitos_clase_Amigo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROGRAMACION\SG_Regional_Conquis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROGRAMACION\SG_Regional_Conquis\Archivos Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{950CEE9D-F433-4DA0-BDF8-D6354A324B2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F45D753E-FD60-4BEE-902C-8CDD0C64B60E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Regular" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="55">
   <si>
     <t>claseId</t>
   </si>
@@ -44,12 +44,6 @@
   </si>
   <si>
     <t>opcionesExtra</t>
-  </si>
-  <si>
-    <t>requiereFoto</t>
-  </si>
-  <si>
-    <t>puntosXp</t>
   </si>
   <si>
     <t>I. Generales</t>
@@ -95,11 +89,6 @@
     <t>1. Dedicar dos horas ayudando a alguien en su comunidad a través de dos de las siguientes actividades:</t>
   </si>
   <si>
-    <t>a) Visitar a alguien que necesita de amistad y orar con esa persona.
-b) Ofrecer y llevar alimento a alguien necesitado.
-c) Participar de un proyecto ecológico o educativo.</t>
-  </si>
-  <si>
     <t>2. Escribir una redacción de cómo ser un buen ciudadano en el hogar y en la escuela</t>
   </si>
   <si>
@@ -118,101 +107,98 @@
     <t>1. Completar una de las siguientes especialidades:</t>
   </si>
   <si>
-    <t>a) Natación I
-b) Educación física
-c) Nudos</t>
+    <t>3. Aprender los principios de una dieta saludable y ayudar a preparar un cuadro con los grupos básicos de alimentos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VI. Organización y liderazgo </t>
+  </si>
+  <si>
+    <t>1. A través de la observación, acompañar todo el proceso del planeamiento hasta la ejecución de una caminata de 5 km.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VII. Estudio de la naturaleza </t>
+  </si>
+  <si>
+    <t>1. Demostrar cómo cuidar correctamente de una cuerda. Hacer y explicar el uso práctico de los siguientes nudos: Simple o Cote; Falso; Verdadero o Llano; Cirujano; As de guía; As de guía doble; Vuelta de escota; Margarita; Pescador; Ancla; Ballestrinque; Vuelta de gancho; Leñador; Grupo de calabrote</t>
+  </si>
+  <si>
+    <t>2. Aprender y demostrar una forma para purificar el agua y escribir un párrafo destacando el significado de Jesús como el Agua de Vida.</t>
+  </si>
+  <si>
+    <t>3. Aprender y armar una tienda de campaña en un lugar apropiado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VIII. Arte de acampar </t>
+  </si>
+  <si>
+    <t>3. Presentar en forma escrita diez reglas para una caminata y explicar qué hacer en caso que esté perdido.</t>
+  </si>
+  <si>
+    <t>4. Aprender las señales para seguir una pista. Prepara y seguir una pista con un mínimo de diez señales que también pueda ser seguida por otros.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IX. Estilo de vida </t>
+  </si>
+  <si>
+    <t>1. Completar una especialidad en el área de Artes y actividades manuales.</t>
+  </si>
+  <si>
+    <t>1. Memorizar, cantar o tocar el Himno de los Conquistadores y conocer la historia del himno.</t>
+  </si>
+  <si>
+    <t>2. En consulta con su líder, escoger uno de los siguientes personajes del Antiguo Testamento y conversar con su grupo sobre el amor y cuidado de Dios y la liberación demostrada en la vida del personaje escogido.</t>
+  </si>
+  <si>
+    <t>3. Llevar por lo menos dos amigos no adventistas a la Escuela Sabática o al Club de Conquistadores.</t>
+  </si>
+  <si>
+    <t>4. Conocer los principios de higiene, buenos modales en la mesa y el comportamiento delante de personas de diferentes edades. Demostrar y explicar cómo estos buenos modales pueden ser útiles en las reuniones y campamentos del club.</t>
+  </si>
+  <si>
+    <t>5. Realizar la especialidad de Arte de acampar.</t>
+  </si>
+  <si>
+    <t>6. Conocer e identificar diez flores silvestres y diez insectos de su región.</t>
+  </si>
+  <si>
+    <t>7. Hacer una fogata utilizando materiales naturales y mantenerla encendida.</t>
+  </si>
+  <si>
+    <t>8. Usar correctamente un cuchillo, un machete o un hacha, y conocer diez reglas para usarlos con seguridad.</t>
+  </si>
+  <si>
+    <t>9. Escoger y completar una especialidad de una de las siguientes áreas:</t>
+  </si>
+  <si>
+    <t>CATEGORIA:ARTES Y HABILIDADES MANUALES</t>
+  </si>
+  <si>
+    <t>OPCIONES:José|Jonás|Ester|Rut</t>
+  </si>
+  <si>
+    <t>observaciones</t>
   </si>
   <si>
     <t>2. Utilizando la experiencia de Daniel:
-     a) Explicar los principios de temperancia que él defendió, o participar de una presentación o escenificación de Daniel 1.
+     a) Explicar los principios de temperancia que él defendió, o participar de una presentación o escenificación de Daniel.
      b) Memorizar y explicar Daniel 1:8.
      c) Escribir su compromiso personal de seguir un estilo de vida saludable.</t>
   </si>
   <si>
-    <t>3. Aprender los principios de una dieta saludable y ayudar a preparar un cuadro con los grupos básicos de alimentos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VI. Organización y liderazgo </t>
-  </si>
-  <si>
-    <t>1. A través de la observación, acompañar todo el proceso del planeamiento hasta la ejecución de una caminata de 5 km.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VII. Estudio de la naturaleza </t>
-  </si>
-  <si>
-    <t>1. Demostrar cómo cuidar correctamente de una cuerda. Hacer y explicar el uso práctico de los siguientes nudos: Simple o Cote; Falso; Verdadero o Llano; Cirujano; As de guía; As de guía doble; Vuelta de escota; Margarita; Pescador; Ancla; Ballestrinque; Vuelta de gancho; Leñador; Grupo de calabrote</t>
-  </si>
-  <si>
-    <t>2. Completar la especialidad de Campamento I.</t>
-  </si>
-  <si>
-    <t>a) Gatos
-b) Perros
-c) Mamíferos
-d) Semillas
-e) Aves de jaula</t>
-  </si>
-  <si>
-    <t>2. Aprender y demostrar una forma para purificar el agua y escribir un párrafo destacando el significado de Jesús como el Agua de Vida.</t>
-  </si>
-  <si>
-    <t>3. Aprender y armar una tienda de campaña en un lugar apropiado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VIII. Arte de acampar </t>
-  </si>
-  <si>
-    <t>3. Presentar en forma escrita diez reglas para una caminata y explicar qué hacer en caso que esté perdido.</t>
-  </si>
-  <si>
-    <t>4. Aprender las señales para seguir una pista. Prepara y seguir una pista con un mínimo de diez señales que también pueda ser seguida por otros.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IX. Estilo de vida </t>
-  </si>
-  <si>
-    <t>1. Completar una especialidad en el área de Artes y actividades manuales.</t>
-  </si>
-  <si>
-    <t>ELEGIR_ESPECIALIDAD_CATEGORIA</t>
-  </si>
-  <si>
-    <t>1. Memorizar, cantar o tocar el Himno de los Conquistadores y conocer la historia del himno.</t>
-  </si>
-  <si>
-    <t>2. En consulta con su líder, escoger uno de los siguientes personajes del Antiguo Testamento y conversar con su grupo sobre el amor y cuidado de Dios y la liberación demostrada en la vida del personaje escogido.</t>
-  </si>
-  <si>
-    <t>a) José
-b) Jonás
-c) Ester
-d) Rut</t>
-  </si>
-  <si>
-    <t>3. Llevar por lo menos dos amigos no adventistas a la Escuela Sabática o al Club de Conquistadores.</t>
-  </si>
-  <si>
-    <t>4. Conocer los principios de higiene, buenos modales en la mesa y el comportamiento delante de personas de diferentes edades. Demostrar y explicar cómo estos buenos modales pueden ser útiles en las reuniones y campamentos del club.</t>
-  </si>
-  <si>
-    <t>5. Realizar la especialidad de Arte de acampar.</t>
-  </si>
-  <si>
-    <t>6. Conocer e identificar diez flores silvestres y diez insectos de su región.</t>
-  </si>
-  <si>
-    <t>7. Hacer una fogata utilizando materiales naturales y mantenerla encendida.</t>
-  </si>
-  <si>
-    <t>8. Usar correctamente un cuchillo, un machete o un hacha, y conocer diez reglas para usarlos con seguridad.</t>
-  </si>
-  <si>
-    <t>9. Escoger y completar una especialidad de una de las siguientes áreas:</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> a) Crecimiento espiritual, actividades misioneras y herencia
- b) Actividades agropecuarias</t>
+    <t>2. Completar la especialidad de Arte de Acampar.</t>
+  </si>
+  <si>
+    <t>CATEGORIA:ACTIVIDADES MISIONERAS Y COMUNITARIAS|ACTIVIDADES AGRÍCOLAS</t>
+  </si>
+  <si>
+    <t>ESPECIALIDADES:Natación I|Educación física|Nudos y amarras|Seguridad básica
+en el agua</t>
+  </si>
+  <si>
+    <t>ESPECIALIDADES:Felinos|Perros|Mamíferos|Semillas|Aves domésticas</t>
+  </si>
+  <si>
+    <t>OPCIONES:Visitar a alguien que necesita de amistad y orar con esa persona|Ofrecer y llevar alimento a alguien necesitado|Participar de un proyecto ecológico o educativo</t>
   </si>
 </sst>
 </file>
@@ -319,7 +305,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -332,7 +318,10 @@
   </cellStyles>
   <dxfs count="16">
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -354,10 +343,10 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -420,7 +409,7 @@
         <name val="Arial"/>
         <scheme val="minor"/>
       </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -456,7 +445,25 @@
         <name val="Arial"/>
         <scheme val="minor"/>
       </font>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -493,42 +500,6 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -583,30 +554,30 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{43BEA4DF-1F83-4520-9428-C8D21711B892}" name="Amigo" displayName="Amigo" ref="A1:H26" totalsRowShown="0" headerRowDxfId="15" dataDxfId="9">
-  <autoFilter ref="A1:H26" xr:uid="{43BEA4DF-1F83-4520-9428-C8D21711B892}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{3AAEB8CD-EF9B-4684-A36D-B3420FFF1D05}" name="claseId" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{6572AA42-4CFE-4232-8BD9-7A9421F18AB0}" name="seccionTitulo" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{EE3647F4-6C02-47FC-83BC-D58143FF0469}" name="ordenSeccion" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{33ED1563-325F-4114-9F22-10D6011DE1EF}" name="numero" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{214C062B-3ECF-4913-8FF3-7A490DBECB6B}" name="descripcion" dataDxfId="10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{43BEA4DF-1F83-4520-9428-C8D21711B892}" name="Amigo" displayName="Amigo" ref="A1:G26" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+  <autoFilter ref="A1:G26" xr:uid="{43BEA4DF-1F83-4520-9428-C8D21711B892}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{3AAEB8CD-EF9B-4684-A36D-B3420FFF1D05}" name="claseId" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{6572AA42-4CFE-4232-8BD9-7A9421F18AB0}" name="seccionTitulo" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{EE3647F4-6C02-47FC-83BC-D58143FF0469}" name="ordenSeccion" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{33ED1563-325F-4114-9F22-10D6011DE1EF}" name="numero" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{214C062B-3ECF-4913-8FF3-7A490DBECB6B}" name="descripcion" dataDxfId="9"/>
     <tableColumn id="6" xr3:uid="{E9D6BFC3-029E-46B1-A302-D7112CEB09F9}" name="opcionesExtra" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{F1D006BA-F5D7-4696-9BBD-14B803009DE6}" name="requiereFoto" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{80904D4C-48C0-4F4B-9F0B-4DAC5B067E77}" name="puntosXp" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{F1D006BA-F5D7-4696-9BBD-14B803009DE6}" name="observaciones" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BD66CA4C-EA80-49C3-B4D0-D0E0756A3C2E}" name="AmigoDeLaNaturaleza" displayName="AmigoDeLaNaturaleza" ref="A1:D10" totalsRowShown="0" headerRowDxfId="5" dataDxfId="3">
-  <autoFilter ref="A1:D10" xr:uid="{BD66CA4C-EA80-49C3-B4D0-D0E0756A3C2E}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{4914C9A0-B031-4FB0-A01C-2D48F35DB49D}" name="claseId" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{E6491CFE-996A-4DD6-9C2B-BF59A15DE057}" name="numero" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{4D1B9C8E-AB05-4925-BA79-9D546BC10BAF}" name="descripcion" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{DE3EF544-2B6A-4C7C-9436-2D34C26FE4D3}" name="opcionesExtra" dataDxfId="4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BD66CA4C-EA80-49C3-B4D0-D0E0756A3C2E}" name="AmigoDeLaNaturaleza" displayName="AmigoDeLaNaturaleza" ref="A1:E10" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+  <autoFilter ref="A1:E10" xr:uid="{BD66CA4C-EA80-49C3-B4D0-D0E0756A3C2E}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{4914C9A0-B031-4FB0-A01C-2D48F35DB49D}" name="claseId" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{E6491CFE-996A-4DD6-9C2B-BF59A15DE057}" name="numero" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{4D1B9C8E-AB05-4925-BA79-9D546BC10BAF}" name="descripcion" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{DE3EF544-2B6A-4C7C-9436-2D34C26FE4D3}" name="opcionesExtra" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{3181BD8D-D033-4BC6-82EE-82156214831E}" name="observaciones" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -813,7 +784,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.140625" customWidth="1"/>
@@ -822,11 +793,10 @@
     <col min="4" max="4" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="80.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="37.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -846,17 +816,16 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2" t="s">
-        <v>8</v>
-      </c>
       <c r="C2" s="3">
         <v>1</v>
       </c>
@@ -864,18 +833,17 @@
         <v>1</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F2" s="6"/>
       <c r="G2" s="5"/>
-      <c r="H2" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A3" s="2"/>
+    </row>
+    <row r="3" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A3" s="3">
+        <v>1</v>
+      </c>
       <c r="B3" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C3" s="3">
         <v>1</v>
@@ -884,18 +852,17 @@
         <v>2</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="3"/>
-      <c r="H3" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A4" s="2"/>
+    </row>
+    <row r="4" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A4" s="3">
+        <v>1</v>
+      </c>
       <c r="B4" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C4" s="3">
         <v>1</v>
@@ -904,18 +871,17 @@
         <v>3</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="3"/>
-      <c r="H4" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="2"/>
+    </row>
+    <row r="5" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="3">
+        <v>1</v>
+      </c>
       <c r="B5" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C5" s="3">
         <v>1</v>
@@ -924,18 +890,17 @@
         <v>4</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="3"/>
-      <c r="H5" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="15" x14ac:dyDescent="0.2">
-      <c r="A6" s="2"/>
+    </row>
+    <row r="6" spans="1:7" ht="15" x14ac:dyDescent="0.2">
+      <c r="A6" s="3">
+        <v>1</v>
+      </c>
       <c r="B6" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C6" s="3">
         <v>1</v>
@@ -944,18 +909,17 @@
         <v>5</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="3"/>
-      <c r="H6" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="2"/>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="3">
+        <v>1</v>
+      </c>
       <c r="B7" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C7" s="3">
         <v>1</v>
@@ -964,18 +928,17 @@
         <v>6</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="3"/>
-      <c r="H7" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="95.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="2"/>
+    </row>
+    <row r="8" spans="1:7" ht="95.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="3">
+        <v>1</v>
+      </c>
       <c r="B8" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C8" s="3">
         <v>2</v>
@@ -984,18 +947,17 @@
         <v>1</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F8" s="10"/>
       <c r="G8" s="3"/>
-      <c r="H8" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="2"/>
+    </row>
+    <row r="9" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="3">
+        <v>1</v>
+      </c>
       <c r="B9" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C9" s="3">
         <v>2</v>
@@ -1004,18 +966,17 @@
         <v>2</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="3"/>
-      <c r="H9" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="9"/>
+    </row>
+    <row r="10" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
+        <v>1</v>
+      </c>
       <c r="B10" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C10" s="5">
         <v>2</v>
@@ -1024,18 +985,17 @@
         <v>3</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F10" s="9"/>
       <c r="G10" s="5"/>
-      <c r="H10" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="76.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="9"/>
+    </row>
+    <row r="11" spans="1:7" ht="63.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
+        <v>1</v>
+      </c>
       <c r="B11" s="8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C11" s="5">
         <v>3</v>
@@ -1044,20 +1004,19 @@
         <v>1</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="G11" s="5"/>
-      <c r="H11" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="9"/>
+    </row>
+    <row r="12" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
+        <v>1</v>
+      </c>
       <c r="B12" s="8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C12" s="5">
         <v>3</v>
@@ -1066,18 +1025,17 @@
         <v>2</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F12" s="9"/>
       <c r="G12" s="5"/>
-      <c r="H12" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="9"/>
+    </row>
+    <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
+        <v>1</v>
+      </c>
       <c r="B13" s="8" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C13" s="5">
         <v>4</v>
@@ -1086,18 +1044,17 @@
         <v>1</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F13" s="9"/>
       <c r="G13" s="5"/>
-      <c r="H13" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="9"/>
+    </row>
+    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
+        <v>1</v>
+      </c>
       <c r="B14" s="8" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C14" s="5">
         <v>4</v>
@@ -1106,18 +1063,17 @@
         <v>2</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F14" s="9"/>
       <c r="G14" s="5"/>
-      <c r="H14" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A15" s="9"/>
+    </row>
+    <row r="15" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
+        <v>1</v>
+      </c>
       <c r="B15" s="8" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C15" s="5">
         <v>5</v>
@@ -1126,20 +1082,19 @@
         <v>1</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="G15" s="5"/>
-      <c r="H15" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="63.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="9"/>
+    </row>
+    <row r="16" spans="1:7" ht="63.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
+        <v>1</v>
+      </c>
       <c r="B16" s="8" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C16" s="5">
         <v>5</v>
@@ -1148,18 +1103,17 @@
         <v>2</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="F16" s="9"/>
       <c r="G16" s="5"/>
-      <c r="H16" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="9"/>
+    </row>
+    <row r="17" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
+        <v>1</v>
+      </c>
       <c r="B17" s="8" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C17" s="5">
         <v>5</v>
@@ -1168,18 +1122,17 @@
         <v>3</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F17" s="9"/>
       <c r="G17" s="5"/>
-      <c r="H17" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="9"/>
+    </row>
+    <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="3">
+        <v>1</v>
+      </c>
       <c r="B18" s="8" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C18" s="5">
         <v>6</v>
@@ -1188,18 +1141,17 @@
         <v>1</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="F18" s="9"/>
       <c r="G18" s="5"/>
-      <c r="H18" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="63.75" x14ac:dyDescent="0.2">
-      <c r="A19" s="9"/>
+    </row>
+    <row r="19" spans="1:7" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A19" s="3">
+        <v>1</v>
+      </c>
       <c r="B19" s="7" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C19" s="5">
         <v>7</v>
@@ -1208,20 +1160,19 @@
         <v>1</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="G19" s="5"/>
-      <c r="H19" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="30" x14ac:dyDescent="0.2">
-      <c r="A20" s="9"/>
+    </row>
+    <row r="20" spans="1:7" ht="30" x14ac:dyDescent="0.2">
+      <c r="A20" s="3">
+        <v>1</v>
+      </c>
       <c r="B20" s="7" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C20" s="5">
         <v>7</v>
@@ -1230,18 +1181,17 @@
         <v>2</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="F20" s="10"/>
       <c r="G20" s="5"/>
-      <c r="H20" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="9"/>
+    </row>
+    <row r="21" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="3">
+        <v>1</v>
+      </c>
       <c r="B21" s="7" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C21" s="5">
         <v>7</v>
@@ -1250,18 +1200,17 @@
         <v>3</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="F21" s="9"/>
       <c r="G21" s="5"/>
-      <c r="H21" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="60" x14ac:dyDescent="0.25">
-      <c r="A22" s="9"/>
+    </row>
+    <row r="22" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A22" s="3">
+        <v>1</v>
+      </c>
       <c r="B22" s="8" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C22" s="5">
         <v>8</v>
@@ -1270,18 +1219,17 @@
         <v>1</v>
       </c>
       <c r="E22" s="11" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="F22" s="9"/>
       <c r="G22" s="5"/>
-      <c r="H22" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="A23" s="9"/>
+    </row>
+    <row r="23" spans="1:7" ht="15" x14ac:dyDescent="0.25">
+      <c r="A23" s="3">
+        <v>1</v>
+      </c>
       <c r="B23" s="8" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C23" s="5">
         <v>8</v>
@@ -1290,18 +1238,17 @@
         <v>2</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="F23" s="9"/>
       <c r="G23" s="5"/>
-      <c r="H23" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="9"/>
+    </row>
+    <row r="24" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="3">
+        <v>1</v>
+      </c>
       <c r="B24" s="8" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C24" s="5">
         <v>8</v>
@@ -1310,18 +1257,17 @@
         <v>3</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="F24" s="9"/>
       <c r="G24" s="5"/>
-      <c r="H24" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="9"/>
+    </row>
+    <row r="25" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="3">
+        <v>1</v>
+      </c>
       <c r="B25" s="8" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C25" s="5">
         <v>8</v>
@@ -1330,18 +1276,17 @@
         <v>4</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="F25" s="9"/>
       <c r="G25" s="5"/>
-      <c r="H25" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="9"/>
+    </row>
+    <row r="26" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="3">
+        <v>1</v>
+      </c>
       <c r="B26" s="8" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="C26" s="5">
         <v>9</v>
@@ -1350,15 +1295,12 @@
         <v>1</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G26" s="5"/>
-      <c r="H26" s="5">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1371,14 +1313,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD3012B8-0581-43D2-A429-5E5B7E93D5DC}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="79.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.140625" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -1391,105 +1334,136 @@
       <c r="D1" s="13" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="6"/>
+      <c r="E1" s="13" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="15">
+        <v>7</v>
+      </c>
       <c r="B2" s="15">
         <v>1</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="D2" s="6"/>
-    </row>
-    <row r="3" spans="1:4" ht="51" x14ac:dyDescent="0.2">
-      <c r="A3" s="6"/>
+      <c r="E2" s="6"/>
+    </row>
+    <row r="3" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A3" s="15">
+        <v>7</v>
+      </c>
       <c r="B3" s="15">
         <v>2</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="30" x14ac:dyDescent="0.2">
-      <c r="A4" s="6"/>
+      <c r="E3" s="14"/>
+    </row>
+    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.2">
+      <c r="A4" s="15">
+        <v>7</v>
+      </c>
       <c r="B4" s="15">
         <v>3</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="D4" s="6"/>
-    </row>
-    <row r="5" spans="1:4" ht="45" x14ac:dyDescent="0.2">
-      <c r="A5" s="6"/>
+      <c r="E4" s="6"/>
+    </row>
+    <row r="5" spans="1:5" ht="45" x14ac:dyDescent="0.2">
+      <c r="A5" s="15">
+        <v>7</v>
+      </c>
       <c r="B5" s="15">
         <v>4</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="D5" s="6"/>
-    </row>
-    <row r="6" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A6" s="6"/>
+      <c r="E5" s="6"/>
+    </row>
+    <row r="6" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A6" s="15">
+        <v>7</v>
+      </c>
       <c r="B6" s="15">
         <v>5</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="D6" s="6"/>
-    </row>
-    <row r="7" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A7" s="6"/>
+      <c r="E6" s="6"/>
+    </row>
+    <row r="7" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A7" s="15">
+        <v>7</v>
+      </c>
       <c r="B7" s="15">
         <v>6</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="D7" s="6"/>
-    </row>
-    <row r="8" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A8" s="6"/>
+      <c r="E7" s="6"/>
+    </row>
+    <row r="8" spans="1:5" ht="15" x14ac:dyDescent="0.2">
+      <c r="A8" s="15">
+        <v>7</v>
+      </c>
       <c r="B8" s="15">
         <v>7</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="D8" s="6"/>
-    </row>
-    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.2">
-      <c r="A9" s="6"/>
+      <c r="E8" s="6"/>
+    </row>
+    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.2">
+      <c r="A9" s="15">
+        <v>7</v>
+      </c>
       <c r="B9" s="15">
         <v>8</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="D9" s="6"/>
-    </row>
-    <row r="10" spans="1:4" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A10" s="6"/>
+      <c r="E9" s="6"/>
+    </row>
+    <row r="10" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A10" s="15">
+        <v>7</v>
+      </c>
       <c r="B10" s="15">
         <v>9</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>55</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="E10" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>